<commit_message>
corregi bug al subir archivo al drive, falta testing, falta crud de drive y listXlsx,
</commit_message>
<xml_diff>
--- a/LISTAS/mi/SOPORTE para CORTINA LIDIMA.xlsx
+++ b/LISTAS/mi/SOPORTE para CORTINA LIDIMA.xlsx
@@ -809,7 +809,7 @@
       </c>
       <c r="C29" s="27" t="n"/>
       <c r="D29" s="15" t="n">
-        <v>113.01</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30" ht="19.5" customHeight="1" s="1">
@@ -987,8 +987,8 @@
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="B30:C30"/>
+    <mergeCell ref="A9:D9"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A9:D9"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B37:C37"/>

</xml_diff>